<commit_message>
RF05c: aguarda recusa transitória no preparo dos cenários
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/matching.xlsx
+++ b/frontend/runner/exemplos/matching.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="104">
   <si>
     <t>cenario</t>
   </si>
@@ -813,11 +813,11 @@
       <c r="I2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" t="s">
-        <v>18</v>
+      <c r="J2">
+        <v>200</v>
+      </c>
+      <c r="K2">
+        <v>15000</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -848,11 +848,11 @@
       <c r="I3" t="s">
         <v>18</v>
       </c>
-      <c r="J3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" t="s">
-        <v>18</v>
+      <c r="J3">
+        <v>200</v>
+      </c>
+      <c r="K3">
+        <v>15000</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1268,11 +1268,11 @@
       <c r="I15" t="s">
         <v>18</v>
       </c>
-      <c r="J15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K15" t="s">
-        <v>18</v>
+      <c r="J15">
+        <v>200</v>
+      </c>
+      <c r="K15">
+        <v>15000</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1303,11 +1303,11 @@
       <c r="I16" t="s">
         <v>18</v>
       </c>
-      <c r="J16" t="s">
-        <v>18</v>
-      </c>
-      <c r="K16" t="s">
-        <v>18</v>
+      <c r="J16">
+        <v>200</v>
+      </c>
+      <c r="K16">
+        <v>15000</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1723,11 +1723,11 @@
       <c r="I28" t="s">
         <v>18</v>
       </c>
-      <c r="J28" t="s">
-        <v>18</v>
-      </c>
-      <c r="K28" t="s">
-        <v>18</v>
+      <c r="J28">
+        <v>200</v>
+      </c>
+      <c r="K28">
+        <v>15000</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1758,11 +1758,11 @@
       <c r="I29" t="s">
         <v>18</v>
       </c>
-      <c r="J29" t="s">
-        <v>18</v>
-      </c>
-      <c r="K29" t="s">
-        <v>18</v>
+      <c r="J29">
+        <v>200</v>
+      </c>
+      <c r="K29">
+        <v>15000</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
RF05c.3b2 (em andamento): MO admite par OCO v3, API expõe redução e matching.xlsx ganha cenários OCO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/matching.xlsx
+++ b/frontend/runner/exemplos/matching.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2091" uniqueCount="289">
   <si>
     <t>cenario</t>
   </si>
@@ -567,6 +567,183 @@
     <t>SemReservasInvalidas</t>
   </si>
   <si>
+    <t>OcoAlvoExecutaCancelaStop</t>
+  </si>
+  <si>
+    <t>Oco</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens-oco</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-Oco"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"VENDA","quantidade":2,"validade":"DIA","takeProfit":{"precoLimite":"10.20"},"stopLoss":{"tipo":"STOP","precoGatilho":"9.80"}}</t>
+  </si>
+  <si>
+    <t>{"Oco":"/grupoOco"}</t>
+  </si>
+  <si>
+    <t>OcoAdmitido</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens-oco/${Oco}</t>
+  </si>
+  <si>
+    <t>CustodiaReservadaUmaVez</t>
+  </si>
+  <si>
+    <t>CompraAlvo</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-CompraAlvo"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"IOC","quantidade":2,"precoLimite":"10.20"}</t>
+  </si>
+  <si>
+    <t>{"CompraAlvo":"/id"}</t>
+  </si>
+  <si>
+    <t>CompraAlvoExecutada</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${CompraAlvo}</t>
+  </si>
+  <si>
+    <t>OcoEncerrado</t>
+  </si>
+  <si>
+    <t>CaixaFinalOcoAlvo</t>
+  </si>
+  <si>
+    <t>CustodiaFinalOcoAlvo</t>
+  </si>
+  <si>
+    <t>OcoParcialReduzStopEGatilhoCancelaAlvo</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"VENDA","quantidade":3,"validade":"DIA","takeProfit":{"precoLimite":"10.20"},"stopLoss":{"tipo":"STOP","precoGatilho":"9.90"}}</t>
+  </si>
+  <si>
+    <t>CompraParcial</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-CompraParcial"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"IOC","quantidade":1,"precoLimite":"10.20"}</t>
+  </si>
+  <si>
+    <t>{"CompraParcial":"/id"}</t>
+  </si>
+  <si>
+    <t>CompraParcialExecutada</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${CompraParcial}</t>
+  </si>
+  <si>
+    <t>StopReduzido</t>
+  </si>
+  <si>
+    <t>CompraGatilho</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-CompraGatilho"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":1,"precoLimite":"9.90"}</t>
+  </si>
+  <si>
+    <t>{"CompraGatilho":"/id"}</t>
+  </si>
+  <si>
+    <t>CompraGatilhoAberta</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${CompraGatilho}</t>
+  </si>
+  <si>
+    <t>LiquidezStop</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-LiquidezStop"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":2,"precoLimite":"9.85"}</t>
+  </si>
+  <si>
+    <t>{"LiquidezStop":"/id"}</t>
+  </si>
+  <si>
+    <t>LiquidezStopAberta</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${LiquidezStop}</t>
+  </si>
+  <si>
+    <t>VendaGatilho</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-VendaGatilho"}</t>
+  </si>
+  <si>
+    <t>{"VendaGatilho":"/id"}</t>
+  </si>
+  <si>
+    <t>VendaGatilhoExecutada</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${VendaGatilho}</t>
+  </si>
+  <si>
+    <t>GatilhoCancelaAlvo</t>
+  </si>
+  <si>
+    <t>LiquidezStopConsumida</t>
+  </si>
+  <si>
+    <t>CaixaFinalOcoStop</t>
+  </si>
+  <si>
+    <t>CustodiaFinalOcoStop</t>
+  </si>
+  <si>
+    <t>OcoCompraAlvoDevolveTroco</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","quantidade":2,"validade":"DIA","takeProfit":{"precoLimite":"9.80"},"stopLoss":{"tipo":"STOP","precoGatilho":"10.20"}}</t>
+  </si>
+  <si>
+    <t>ReservaUnicaPar</t>
+  </si>
+  <si>
+    <t>VendaAlvo</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-VendaAlvo"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"VENDA","tipo":"LIMIT","validade":"IOC","quantidade":2,"precoLimite":"9.80"}</t>
+  </si>
+  <si>
+    <t>{"VendaAlvo":"/id"}</t>
+  </si>
+  <si>
+    <t>VendaAlvoExecutada</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${VendaAlvo}</t>
+  </si>
+  <si>
+    <t>CaixaFinalOcoCompra</t>
+  </si>
+  <si>
+    <t>CustodiaFinalOcoCompra</t>
+  </si>
+  <si>
     <t>passo</t>
   </si>
   <si>
@@ -667,6 +844,42 @@
   </si>
   <si>
     <t>{"/saldoTotal":"960.30","/saldoReservado":"0.00"}</t>
+  </si>
+  <si>
+    <t>{"/ordens/0/papelOco":"TAKE_PROFIT","/ordens/0/estado":"ABERTA","/ordens/1/papelOco":"STOP_LOSS","/ordens/1/estado":"AGUARDANDO_GATILHO"}</t>
+  </si>
+  <si>
+    <t>{"/custodias/0/reservado":2}</t>
+  </si>
+  <si>
+    <t>{"/ordens/0/estado":"EXECUTADA","/ordens/0/quantidadeExecutada":2,"/ordens/1/estado":"CANCELADA","/ordens/1/motivoEncerramento":"CANCELADA_OCO","/ordens/1/quantidadeExecutada":0,"/ordens/1/quantidadeCancelada":2}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"969.60","/saldoDisponivel":"969.60","/saldoReservado":"0.00"}</t>
+  </si>
+  <si>
+    <t>{"/ordens/0/estado":"ABERTA","/ordens/1/estado":"AGUARDANDO_GATILHO"}</t>
+  </si>
+  <si>
+    <t>{"/ordens/0/estado":"PARCIALMENTE_EXECUTADA","/ordens/0/quantidadeExecutada":1,"/ordens/1/estado":"AGUARDANDO_GATILHO","/ordens/1/quantidadeReduzida":1}</t>
+  </si>
+  <si>
+    <t>{"/ordens/0/estado":"CANCELADA","/ordens/0/motivoEncerramento":"CANCELADA_OCO","/ordens/0/quantidadeExecutada":1,"/ordens/0/quantidadeCancelada":2,"/ordens/1/estado":"EXECUTADA","/ordens/1/quantidadeExecutada":2,"/ordens/1/quantidadeReduzida":1}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"950.20","/saldoDisponivel":"950.20","/saldoReservado":"0.00"}</t>
+  </si>
+  <si>
+    <t>{"/custodias/0/total":95,"/custodias/0/reservado":0}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"990.00","/saldoReservado":"22.44"}</t>
+  </si>
+  <si>
+    <t>{"/ordens/0/estado":"EXECUTADA","/ordens/1/estado":"CANCELADA","/ordens/1/motivoEncerramento":"CANCELADA_OCO"}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"970.40","/saldoDisponivel":"970.40","/saldoReservado":"0.00"}</t>
   </si>
 </sst>
 </file>
@@ -1089,7 +1302,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K165"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5044,6 +5257,1826 @@
         <v>200</v>
       </c>
       <c r="K113">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>184</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>12</v>
+      </c>
+      <c r="D114" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>15</v>
+      </c>
+      <c r="G114" t="s">
+        <v>16</v>
+      </c>
+      <c r="H114" t="s">
+        <v>17</v>
+      </c>
+      <c r="I114" t="s">
+        <v>18</v>
+      </c>
+      <c r="J114">
+        <v>200</v>
+      </c>
+      <c r="K114">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>184</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>19</v>
+      </c>
+      <c r="D115" t="s">
+        <v>13</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>20</v>
+      </c>
+      <c r="G115" t="s">
+        <v>16</v>
+      </c>
+      <c r="H115" t="s">
+        <v>17</v>
+      </c>
+      <c r="I115" t="s">
+        <v>18</v>
+      </c>
+      <c r="J115">
+        <v>200</v>
+      </c>
+      <c r="K115">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>184</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>86</v>
+      </c>
+      <c r="D116" t="s">
+        <v>22</v>
+      </c>
+      <c r="E116" t="s">
+        <v>23</v>
+      </c>
+      <c r="F116" t="s">
+        <v>24</v>
+      </c>
+      <c r="G116" t="s">
+        <v>87</v>
+      </c>
+      <c r="H116" t="s">
+        <v>88</v>
+      </c>
+      <c r="I116" t="s">
+        <v>89</v>
+      </c>
+      <c r="J116" t="s">
+        <v>18</v>
+      </c>
+      <c r="K116" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>184</v>
+      </c>
+      <c r="B117">
+        <v>4</v>
+      </c>
+      <c r="C117" t="s">
+        <v>90</v>
+      </c>
+      <c r="D117" t="s">
+        <v>22</v>
+      </c>
+      <c r="E117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F117" t="s">
+        <v>91</v>
+      </c>
+      <c r="G117" t="s">
+        <v>18</v>
+      </c>
+      <c r="H117" t="s">
+        <v>18</v>
+      </c>
+      <c r="I117" t="s">
+        <v>18</v>
+      </c>
+      <c r="J117">
+        <v>200</v>
+      </c>
+      <c r="K117">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>184</v>
+      </c>
+      <c r="B118">
+        <v>5</v>
+      </c>
+      <c r="C118" t="s">
+        <v>92</v>
+      </c>
+      <c r="D118" t="s">
+        <v>40</v>
+      </c>
+      <c r="E118" t="s">
+        <v>23</v>
+      </c>
+      <c r="F118" t="s">
+        <v>24</v>
+      </c>
+      <c r="G118" t="s">
+        <v>93</v>
+      </c>
+      <c r="H118" t="s">
+        <v>94</v>
+      </c>
+      <c r="I118" t="s">
+        <v>95</v>
+      </c>
+      <c r="J118" t="s">
+        <v>18</v>
+      </c>
+      <c r="K118" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>184</v>
+      </c>
+      <c r="B119">
+        <v>6</v>
+      </c>
+      <c r="C119" t="s">
+        <v>96</v>
+      </c>
+      <c r="D119" t="s">
+        <v>40</v>
+      </c>
+      <c r="E119" t="s">
+        <v>29</v>
+      </c>
+      <c r="F119" t="s">
+        <v>97</v>
+      </c>
+      <c r="G119" t="s">
+        <v>18</v>
+      </c>
+      <c r="H119" t="s">
+        <v>18</v>
+      </c>
+      <c r="I119" t="s">
+        <v>18</v>
+      </c>
+      <c r="J119">
+        <v>200</v>
+      </c>
+      <c r="K119">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>184</v>
+      </c>
+      <c r="B120">
+        <v>7</v>
+      </c>
+      <c r="C120" t="s">
+        <v>98</v>
+      </c>
+      <c r="D120" t="s">
+        <v>22</v>
+      </c>
+      <c r="E120" t="s">
+        <v>29</v>
+      </c>
+      <c r="F120" t="s">
+        <v>91</v>
+      </c>
+      <c r="G120" t="s">
+        <v>18</v>
+      </c>
+      <c r="H120" t="s">
+        <v>18</v>
+      </c>
+      <c r="I120" t="s">
+        <v>18</v>
+      </c>
+      <c r="J120">
+        <v>200</v>
+      </c>
+      <c r="K120">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>184</v>
+      </c>
+      <c r="B121">
+        <v>8</v>
+      </c>
+      <c r="C121" t="s">
+        <v>185</v>
+      </c>
+      <c r="D121" t="s">
+        <v>22</v>
+      </c>
+      <c r="E121" t="s">
+        <v>23</v>
+      </c>
+      <c r="F121" t="s">
+        <v>186</v>
+      </c>
+      <c r="G121" t="s">
+        <v>187</v>
+      </c>
+      <c r="H121" t="s">
+        <v>188</v>
+      </c>
+      <c r="I121" t="s">
+        <v>189</v>
+      </c>
+      <c r="J121" t="s">
+        <v>18</v>
+      </c>
+      <c r="K121" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>184</v>
+      </c>
+      <c r="B122">
+        <v>9</v>
+      </c>
+      <c r="C122" t="s">
+        <v>190</v>
+      </c>
+      <c r="D122" t="s">
+        <v>22</v>
+      </c>
+      <c r="E122" t="s">
+        <v>29</v>
+      </c>
+      <c r="F122" t="s">
+        <v>191</v>
+      </c>
+      <c r="G122" t="s">
+        <v>18</v>
+      </c>
+      <c r="H122" t="s">
+        <v>18</v>
+      </c>
+      <c r="I122" t="s">
+        <v>18</v>
+      </c>
+      <c r="J122">
+        <v>200</v>
+      </c>
+      <c r="K122">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>184</v>
+      </c>
+      <c r="B123">
+        <v>10</v>
+      </c>
+      <c r="C123" t="s">
+        <v>192</v>
+      </c>
+      <c r="D123" t="s">
+        <v>52</v>
+      </c>
+      <c r="E123" t="s">
+        <v>29</v>
+      </c>
+      <c r="F123" t="s">
+        <v>50</v>
+      </c>
+      <c r="G123" t="s">
+        <v>18</v>
+      </c>
+      <c r="H123" t="s">
+        <v>18</v>
+      </c>
+      <c r="I123" t="s">
+        <v>18</v>
+      </c>
+      <c r="J123">
+        <v>200</v>
+      </c>
+      <c r="K123">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>184</v>
+      </c>
+      <c r="B124">
+        <v>11</v>
+      </c>
+      <c r="C124" t="s">
+        <v>193</v>
+      </c>
+      <c r="D124" t="s">
+        <v>40</v>
+      </c>
+      <c r="E124" t="s">
+        <v>23</v>
+      </c>
+      <c r="F124" t="s">
+        <v>24</v>
+      </c>
+      <c r="G124" t="s">
+        <v>194</v>
+      </c>
+      <c r="H124" t="s">
+        <v>195</v>
+      </c>
+      <c r="I124" t="s">
+        <v>196</v>
+      </c>
+      <c r="J124" t="s">
+        <v>18</v>
+      </c>
+      <c r="K124" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>184</v>
+      </c>
+      <c r="B125">
+        <v>12</v>
+      </c>
+      <c r="C125" t="s">
+        <v>197</v>
+      </c>
+      <c r="D125" t="s">
+        <v>40</v>
+      </c>
+      <c r="E125" t="s">
+        <v>29</v>
+      </c>
+      <c r="F125" t="s">
+        <v>198</v>
+      </c>
+      <c r="G125" t="s">
+        <v>18</v>
+      </c>
+      <c r="H125" t="s">
+        <v>18</v>
+      </c>
+      <c r="I125" t="s">
+        <v>18</v>
+      </c>
+      <c r="J125">
+        <v>200</v>
+      </c>
+      <c r="K125">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>184</v>
+      </c>
+      <c r="B126">
+        <v>13</v>
+      </c>
+      <c r="C126" t="s">
+        <v>199</v>
+      </c>
+      <c r="D126" t="s">
+        <v>22</v>
+      </c>
+      <c r="E126" t="s">
+        <v>29</v>
+      </c>
+      <c r="F126" t="s">
+        <v>191</v>
+      </c>
+      <c r="G126" t="s">
+        <v>18</v>
+      </c>
+      <c r="H126" t="s">
+        <v>18</v>
+      </c>
+      <c r="I126" t="s">
+        <v>18</v>
+      </c>
+      <c r="J126">
+        <v>200</v>
+      </c>
+      <c r="K126">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>184</v>
+      </c>
+      <c r="B127">
+        <v>14</v>
+      </c>
+      <c r="C127" t="s">
+        <v>200</v>
+      </c>
+      <c r="D127" t="s">
+        <v>49</v>
+      </c>
+      <c r="E127" t="s">
+        <v>29</v>
+      </c>
+      <c r="F127" t="s">
+        <v>50</v>
+      </c>
+      <c r="G127" t="s">
+        <v>18</v>
+      </c>
+      <c r="H127" t="s">
+        <v>18</v>
+      </c>
+      <c r="I127" t="s">
+        <v>18</v>
+      </c>
+      <c r="J127">
+        <v>200</v>
+      </c>
+      <c r="K127">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>184</v>
+      </c>
+      <c r="B128">
+        <v>15</v>
+      </c>
+      <c r="C128" t="s">
+        <v>201</v>
+      </c>
+      <c r="D128" t="s">
+        <v>52</v>
+      </c>
+      <c r="E128" t="s">
+        <v>29</v>
+      </c>
+      <c r="F128" t="s">
+        <v>50</v>
+      </c>
+      <c r="G128" t="s">
+        <v>18</v>
+      </c>
+      <c r="H128" t="s">
+        <v>18</v>
+      </c>
+      <c r="I128" t="s">
+        <v>18</v>
+      </c>
+      <c r="J128">
+        <v>200</v>
+      </c>
+      <c r="K128">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>202</v>
+      </c>
+      <c r="B129">
+        <v>1</v>
+      </c>
+      <c r="C129" t="s">
+        <v>12</v>
+      </c>
+      <c r="D129" t="s">
+        <v>13</v>
+      </c>
+      <c r="E129" t="s">
+        <v>14</v>
+      </c>
+      <c r="F129" t="s">
+        <v>15</v>
+      </c>
+      <c r="G129" t="s">
+        <v>16</v>
+      </c>
+      <c r="H129" t="s">
+        <v>17</v>
+      </c>
+      <c r="I129" t="s">
+        <v>18</v>
+      </c>
+      <c r="J129">
+        <v>200</v>
+      </c>
+      <c r="K129">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>202</v>
+      </c>
+      <c r="B130">
+        <v>2</v>
+      </c>
+      <c r="C130" t="s">
+        <v>19</v>
+      </c>
+      <c r="D130" t="s">
+        <v>13</v>
+      </c>
+      <c r="E130" t="s">
+        <v>14</v>
+      </c>
+      <c r="F130" t="s">
+        <v>20</v>
+      </c>
+      <c r="G130" t="s">
+        <v>16</v>
+      </c>
+      <c r="H130" t="s">
+        <v>17</v>
+      </c>
+      <c r="I130" t="s">
+        <v>18</v>
+      </c>
+      <c r="J130">
+        <v>200</v>
+      </c>
+      <c r="K130">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>202</v>
+      </c>
+      <c r="B131">
+        <v>3</v>
+      </c>
+      <c r="C131" t="s">
+        <v>86</v>
+      </c>
+      <c r="D131" t="s">
+        <v>22</v>
+      </c>
+      <c r="E131" t="s">
+        <v>23</v>
+      </c>
+      <c r="F131" t="s">
+        <v>24</v>
+      </c>
+      <c r="G131" t="s">
+        <v>87</v>
+      </c>
+      <c r="H131" t="s">
+        <v>88</v>
+      </c>
+      <c r="I131" t="s">
+        <v>89</v>
+      </c>
+      <c r="J131" t="s">
+        <v>18</v>
+      </c>
+      <c r="K131" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>202</v>
+      </c>
+      <c r="B132">
+        <v>4</v>
+      </c>
+      <c r="C132" t="s">
+        <v>90</v>
+      </c>
+      <c r="D132" t="s">
+        <v>22</v>
+      </c>
+      <c r="E132" t="s">
+        <v>29</v>
+      </c>
+      <c r="F132" t="s">
+        <v>91</v>
+      </c>
+      <c r="G132" t="s">
+        <v>18</v>
+      </c>
+      <c r="H132" t="s">
+        <v>18</v>
+      </c>
+      <c r="I132" t="s">
+        <v>18</v>
+      </c>
+      <c r="J132">
+        <v>200</v>
+      </c>
+      <c r="K132">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>202</v>
+      </c>
+      <c r="B133">
+        <v>5</v>
+      </c>
+      <c r="C133" t="s">
+        <v>92</v>
+      </c>
+      <c r="D133" t="s">
+        <v>40</v>
+      </c>
+      <c r="E133" t="s">
+        <v>23</v>
+      </c>
+      <c r="F133" t="s">
+        <v>24</v>
+      </c>
+      <c r="G133" t="s">
+        <v>93</v>
+      </c>
+      <c r="H133" t="s">
+        <v>94</v>
+      </c>
+      <c r="I133" t="s">
+        <v>95</v>
+      </c>
+      <c r="J133" t="s">
+        <v>18</v>
+      </c>
+      <c r="K133" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>202</v>
+      </c>
+      <c r="B134">
+        <v>6</v>
+      </c>
+      <c r="C134" t="s">
+        <v>96</v>
+      </c>
+      <c r="D134" t="s">
+        <v>40</v>
+      </c>
+      <c r="E134" t="s">
+        <v>29</v>
+      </c>
+      <c r="F134" t="s">
+        <v>97</v>
+      </c>
+      <c r="G134" t="s">
+        <v>18</v>
+      </c>
+      <c r="H134" t="s">
+        <v>18</v>
+      </c>
+      <c r="I134" t="s">
+        <v>18</v>
+      </c>
+      <c r="J134">
+        <v>200</v>
+      </c>
+      <c r="K134">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>202</v>
+      </c>
+      <c r="B135">
+        <v>7</v>
+      </c>
+      <c r="C135" t="s">
+        <v>98</v>
+      </c>
+      <c r="D135" t="s">
+        <v>22</v>
+      </c>
+      <c r="E135" t="s">
+        <v>29</v>
+      </c>
+      <c r="F135" t="s">
+        <v>91</v>
+      </c>
+      <c r="G135" t="s">
+        <v>18</v>
+      </c>
+      <c r="H135" t="s">
+        <v>18</v>
+      </c>
+      <c r="I135" t="s">
+        <v>18</v>
+      </c>
+      <c r="J135">
+        <v>200</v>
+      </c>
+      <c r="K135">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>202</v>
+      </c>
+      <c r="B136">
+        <v>8</v>
+      </c>
+      <c r="C136" t="s">
+        <v>185</v>
+      </c>
+      <c r="D136" t="s">
+        <v>22</v>
+      </c>
+      <c r="E136" t="s">
+        <v>23</v>
+      </c>
+      <c r="F136" t="s">
+        <v>186</v>
+      </c>
+      <c r="G136" t="s">
+        <v>187</v>
+      </c>
+      <c r="H136" t="s">
+        <v>203</v>
+      </c>
+      <c r="I136" t="s">
+        <v>189</v>
+      </c>
+      <c r="J136" t="s">
+        <v>18</v>
+      </c>
+      <c r="K136" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>202</v>
+      </c>
+      <c r="B137">
+        <v>9</v>
+      </c>
+      <c r="C137" t="s">
+        <v>190</v>
+      </c>
+      <c r="D137" t="s">
+        <v>22</v>
+      </c>
+      <c r="E137" t="s">
+        <v>29</v>
+      </c>
+      <c r="F137" t="s">
+        <v>191</v>
+      </c>
+      <c r="G137" t="s">
+        <v>18</v>
+      </c>
+      <c r="H137" t="s">
+        <v>18</v>
+      </c>
+      <c r="I137" t="s">
+        <v>18</v>
+      </c>
+      <c r="J137">
+        <v>200</v>
+      </c>
+      <c r="K137">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>202</v>
+      </c>
+      <c r="B138">
+        <v>10</v>
+      </c>
+      <c r="C138" t="s">
+        <v>204</v>
+      </c>
+      <c r="D138" t="s">
+        <v>40</v>
+      </c>
+      <c r="E138" t="s">
+        <v>23</v>
+      </c>
+      <c r="F138" t="s">
+        <v>24</v>
+      </c>
+      <c r="G138" t="s">
+        <v>205</v>
+      </c>
+      <c r="H138" t="s">
+        <v>206</v>
+      </c>
+      <c r="I138" t="s">
+        <v>207</v>
+      </c>
+      <c r="J138" t="s">
+        <v>18</v>
+      </c>
+      <c r="K138" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>202</v>
+      </c>
+      <c r="B139">
+        <v>11</v>
+      </c>
+      <c r="C139" t="s">
+        <v>208</v>
+      </c>
+      <c r="D139" t="s">
+        <v>40</v>
+      </c>
+      <c r="E139" t="s">
+        <v>29</v>
+      </c>
+      <c r="F139" t="s">
+        <v>209</v>
+      </c>
+      <c r="G139" t="s">
+        <v>18</v>
+      </c>
+      <c r="H139" t="s">
+        <v>18</v>
+      </c>
+      <c r="I139" t="s">
+        <v>18</v>
+      </c>
+      <c r="J139">
+        <v>200</v>
+      </c>
+      <c r="K139">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>202</v>
+      </c>
+      <c r="B140">
+        <v>12</v>
+      </c>
+      <c r="C140" t="s">
+        <v>210</v>
+      </c>
+      <c r="D140" t="s">
+        <v>22</v>
+      </c>
+      <c r="E140" t="s">
+        <v>29</v>
+      </c>
+      <c r="F140" t="s">
+        <v>191</v>
+      </c>
+      <c r="G140" t="s">
+        <v>18</v>
+      </c>
+      <c r="H140" t="s">
+        <v>18</v>
+      </c>
+      <c r="I140" t="s">
+        <v>18</v>
+      </c>
+      <c r="J140">
+        <v>200</v>
+      </c>
+      <c r="K140">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>202</v>
+      </c>
+      <c r="B141">
+        <v>13</v>
+      </c>
+      <c r="C141" t="s">
+        <v>211</v>
+      </c>
+      <c r="D141" t="s">
+        <v>40</v>
+      </c>
+      <c r="E141" t="s">
+        <v>23</v>
+      </c>
+      <c r="F141" t="s">
+        <v>24</v>
+      </c>
+      <c r="G141" t="s">
+        <v>212</v>
+      </c>
+      <c r="H141" t="s">
+        <v>213</v>
+      </c>
+      <c r="I141" t="s">
+        <v>214</v>
+      </c>
+      <c r="J141" t="s">
+        <v>18</v>
+      </c>
+      <c r="K141" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>202</v>
+      </c>
+      <c r="B142">
+        <v>14</v>
+      </c>
+      <c r="C142" t="s">
+        <v>215</v>
+      </c>
+      <c r="D142" t="s">
+        <v>40</v>
+      </c>
+      <c r="E142" t="s">
+        <v>29</v>
+      </c>
+      <c r="F142" t="s">
+        <v>216</v>
+      </c>
+      <c r="G142" t="s">
+        <v>18</v>
+      </c>
+      <c r="H142" t="s">
+        <v>18</v>
+      </c>
+      <c r="I142" t="s">
+        <v>18</v>
+      </c>
+      <c r="J142">
+        <v>200</v>
+      </c>
+      <c r="K142">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>202</v>
+      </c>
+      <c r="B143">
+        <v>15</v>
+      </c>
+      <c r="C143" t="s">
+        <v>217</v>
+      </c>
+      <c r="D143" t="s">
+        <v>40</v>
+      </c>
+      <c r="E143" t="s">
+        <v>23</v>
+      </c>
+      <c r="F143" t="s">
+        <v>24</v>
+      </c>
+      <c r="G143" t="s">
+        <v>218</v>
+      </c>
+      <c r="H143" t="s">
+        <v>219</v>
+      </c>
+      <c r="I143" t="s">
+        <v>220</v>
+      </c>
+      <c r="J143" t="s">
+        <v>18</v>
+      </c>
+      <c r="K143" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>202</v>
+      </c>
+      <c r="B144">
+        <v>16</v>
+      </c>
+      <c r="C144" t="s">
+        <v>221</v>
+      </c>
+      <c r="D144" t="s">
+        <v>40</v>
+      </c>
+      <c r="E144" t="s">
+        <v>29</v>
+      </c>
+      <c r="F144" t="s">
+        <v>222</v>
+      </c>
+      <c r="G144" t="s">
+        <v>18</v>
+      </c>
+      <c r="H144" t="s">
+        <v>18</v>
+      </c>
+      <c r="I144" t="s">
+        <v>18</v>
+      </c>
+      <c r="J144">
+        <v>200</v>
+      </c>
+      <c r="K144">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>202</v>
+      </c>
+      <c r="B145">
+        <v>17</v>
+      </c>
+      <c r="C145" t="s">
+        <v>223</v>
+      </c>
+      <c r="D145" t="s">
+        <v>22</v>
+      </c>
+      <c r="E145" t="s">
+        <v>23</v>
+      </c>
+      <c r="F145" t="s">
+        <v>24</v>
+      </c>
+      <c r="G145" t="s">
+        <v>224</v>
+      </c>
+      <c r="H145" t="s">
+        <v>163</v>
+      </c>
+      <c r="I145" t="s">
+        <v>225</v>
+      </c>
+      <c r="J145" t="s">
+        <v>18</v>
+      </c>
+      <c r="K145" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>202</v>
+      </c>
+      <c r="B146">
+        <v>18</v>
+      </c>
+      <c r="C146" t="s">
+        <v>226</v>
+      </c>
+      <c r="D146" t="s">
+        <v>22</v>
+      </c>
+      <c r="E146" t="s">
+        <v>29</v>
+      </c>
+      <c r="F146" t="s">
+        <v>227</v>
+      </c>
+      <c r="G146" t="s">
+        <v>18</v>
+      </c>
+      <c r="H146" t="s">
+        <v>18</v>
+      </c>
+      <c r="I146" t="s">
+        <v>18</v>
+      </c>
+      <c r="J146">
+        <v>200</v>
+      </c>
+      <c r="K146">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>202</v>
+      </c>
+      <c r="B147">
+        <v>19</v>
+      </c>
+      <c r="C147" t="s">
+        <v>228</v>
+      </c>
+      <c r="D147" t="s">
+        <v>22</v>
+      </c>
+      <c r="E147" t="s">
+        <v>29</v>
+      </c>
+      <c r="F147" t="s">
+        <v>191</v>
+      </c>
+      <c r="G147" t="s">
+        <v>18</v>
+      </c>
+      <c r="H147" t="s">
+        <v>18</v>
+      </c>
+      <c r="I147" t="s">
+        <v>18</v>
+      </c>
+      <c r="J147">
+        <v>200</v>
+      </c>
+      <c r="K147">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>202</v>
+      </c>
+      <c r="B148">
+        <v>20</v>
+      </c>
+      <c r="C148" t="s">
+        <v>229</v>
+      </c>
+      <c r="D148" t="s">
+        <v>40</v>
+      </c>
+      <c r="E148" t="s">
+        <v>29</v>
+      </c>
+      <c r="F148" t="s">
+        <v>222</v>
+      </c>
+      <c r="G148" t="s">
+        <v>18</v>
+      </c>
+      <c r="H148" t="s">
+        <v>18</v>
+      </c>
+      <c r="I148" t="s">
+        <v>18</v>
+      </c>
+      <c r="J148">
+        <v>200</v>
+      </c>
+      <c r="K148">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>202</v>
+      </c>
+      <c r="B149">
+        <v>21</v>
+      </c>
+      <c r="C149" t="s">
+        <v>230</v>
+      </c>
+      <c r="D149" t="s">
+        <v>49</v>
+      </c>
+      <c r="E149" t="s">
+        <v>29</v>
+      </c>
+      <c r="F149" t="s">
+        <v>50</v>
+      </c>
+      <c r="G149" t="s">
+        <v>18</v>
+      </c>
+      <c r="H149" t="s">
+        <v>18</v>
+      </c>
+      <c r="I149" t="s">
+        <v>18</v>
+      </c>
+      <c r="J149">
+        <v>200</v>
+      </c>
+      <c r="K149">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>202</v>
+      </c>
+      <c r="B150">
+        <v>22</v>
+      </c>
+      <c r="C150" t="s">
+        <v>231</v>
+      </c>
+      <c r="D150" t="s">
+        <v>52</v>
+      </c>
+      <c r="E150" t="s">
+        <v>29</v>
+      </c>
+      <c r="F150" t="s">
+        <v>50</v>
+      </c>
+      <c r="G150" t="s">
+        <v>18</v>
+      </c>
+      <c r="H150" t="s">
+        <v>18</v>
+      </c>
+      <c r="I150" t="s">
+        <v>18</v>
+      </c>
+      <c r="J150">
+        <v>200</v>
+      </c>
+      <c r="K150">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>232</v>
+      </c>
+      <c r="B151">
+        <v>1</v>
+      </c>
+      <c r="C151" t="s">
+        <v>12</v>
+      </c>
+      <c r="D151" t="s">
+        <v>13</v>
+      </c>
+      <c r="E151" t="s">
+        <v>14</v>
+      </c>
+      <c r="F151" t="s">
+        <v>15</v>
+      </c>
+      <c r="G151" t="s">
+        <v>16</v>
+      </c>
+      <c r="H151" t="s">
+        <v>17</v>
+      </c>
+      <c r="I151" t="s">
+        <v>18</v>
+      </c>
+      <c r="J151">
+        <v>200</v>
+      </c>
+      <c r="K151">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>232</v>
+      </c>
+      <c r="B152">
+        <v>2</v>
+      </c>
+      <c r="C152" t="s">
+        <v>19</v>
+      </c>
+      <c r="D152" t="s">
+        <v>13</v>
+      </c>
+      <c r="E152" t="s">
+        <v>14</v>
+      </c>
+      <c r="F152" t="s">
+        <v>20</v>
+      </c>
+      <c r="G152" t="s">
+        <v>16</v>
+      </c>
+      <c r="H152" t="s">
+        <v>17</v>
+      </c>
+      <c r="I152" t="s">
+        <v>18</v>
+      </c>
+      <c r="J152">
+        <v>200</v>
+      </c>
+      <c r="K152">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>232</v>
+      </c>
+      <c r="B153">
+        <v>3</v>
+      </c>
+      <c r="C153" t="s">
+        <v>86</v>
+      </c>
+      <c r="D153" t="s">
+        <v>22</v>
+      </c>
+      <c r="E153" t="s">
+        <v>23</v>
+      </c>
+      <c r="F153" t="s">
+        <v>24</v>
+      </c>
+      <c r="G153" t="s">
+        <v>87</v>
+      </c>
+      <c r="H153" t="s">
+        <v>88</v>
+      </c>
+      <c r="I153" t="s">
+        <v>89</v>
+      </c>
+      <c r="J153" t="s">
+        <v>18</v>
+      </c>
+      <c r="K153" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>232</v>
+      </c>
+      <c r="B154">
+        <v>4</v>
+      </c>
+      <c r="C154" t="s">
+        <v>90</v>
+      </c>
+      <c r="D154" t="s">
+        <v>22</v>
+      </c>
+      <c r="E154" t="s">
+        <v>29</v>
+      </c>
+      <c r="F154" t="s">
+        <v>91</v>
+      </c>
+      <c r="G154" t="s">
+        <v>18</v>
+      </c>
+      <c r="H154" t="s">
+        <v>18</v>
+      </c>
+      <c r="I154" t="s">
+        <v>18</v>
+      </c>
+      <c r="J154">
+        <v>200</v>
+      </c>
+      <c r="K154">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>232</v>
+      </c>
+      <c r="B155">
+        <v>5</v>
+      </c>
+      <c r="C155" t="s">
+        <v>92</v>
+      </c>
+      <c r="D155" t="s">
+        <v>40</v>
+      </c>
+      <c r="E155" t="s">
+        <v>23</v>
+      </c>
+      <c r="F155" t="s">
+        <v>24</v>
+      </c>
+      <c r="G155" t="s">
+        <v>93</v>
+      </c>
+      <c r="H155" t="s">
+        <v>94</v>
+      </c>
+      <c r="I155" t="s">
+        <v>95</v>
+      </c>
+      <c r="J155" t="s">
+        <v>18</v>
+      </c>
+      <c r="K155" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>232</v>
+      </c>
+      <c r="B156">
+        <v>6</v>
+      </c>
+      <c r="C156" t="s">
+        <v>96</v>
+      </c>
+      <c r="D156" t="s">
+        <v>40</v>
+      </c>
+      <c r="E156" t="s">
+        <v>29</v>
+      </c>
+      <c r="F156" t="s">
+        <v>97</v>
+      </c>
+      <c r="G156" t="s">
+        <v>18</v>
+      </c>
+      <c r="H156" t="s">
+        <v>18</v>
+      </c>
+      <c r="I156" t="s">
+        <v>18</v>
+      </c>
+      <c r="J156">
+        <v>200</v>
+      </c>
+      <c r="K156">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>232</v>
+      </c>
+      <c r="B157">
+        <v>7</v>
+      </c>
+      <c r="C157" t="s">
+        <v>98</v>
+      </c>
+      <c r="D157" t="s">
+        <v>22</v>
+      </c>
+      <c r="E157" t="s">
+        <v>29</v>
+      </c>
+      <c r="F157" t="s">
+        <v>91</v>
+      </c>
+      <c r="G157" t="s">
+        <v>18</v>
+      </c>
+      <c r="H157" t="s">
+        <v>18</v>
+      </c>
+      <c r="I157" t="s">
+        <v>18</v>
+      </c>
+      <c r="J157">
+        <v>200</v>
+      </c>
+      <c r="K157">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>232</v>
+      </c>
+      <c r="B158">
+        <v>8</v>
+      </c>
+      <c r="C158" t="s">
+        <v>185</v>
+      </c>
+      <c r="D158" t="s">
+        <v>40</v>
+      </c>
+      <c r="E158" t="s">
+        <v>23</v>
+      </c>
+      <c r="F158" t="s">
+        <v>186</v>
+      </c>
+      <c r="G158" t="s">
+        <v>187</v>
+      </c>
+      <c r="H158" t="s">
+        <v>233</v>
+      </c>
+      <c r="I158" t="s">
+        <v>189</v>
+      </c>
+      <c r="J158" t="s">
+        <v>18</v>
+      </c>
+      <c r="K158" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>232</v>
+      </c>
+      <c r="B159">
+        <v>9</v>
+      </c>
+      <c r="C159" t="s">
+        <v>190</v>
+      </c>
+      <c r="D159" t="s">
+        <v>40</v>
+      </c>
+      <c r="E159" t="s">
+        <v>29</v>
+      </c>
+      <c r="F159" t="s">
+        <v>191</v>
+      </c>
+      <c r="G159" t="s">
+        <v>18</v>
+      </c>
+      <c r="H159" t="s">
+        <v>18</v>
+      </c>
+      <c r="I159" t="s">
+        <v>18</v>
+      </c>
+      <c r="J159">
+        <v>200</v>
+      </c>
+      <c r="K159">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>232</v>
+      </c>
+      <c r="B160">
+        <v>10</v>
+      </c>
+      <c r="C160" t="s">
+        <v>234</v>
+      </c>
+      <c r="D160" t="s">
+        <v>49</v>
+      </c>
+      <c r="E160" t="s">
+        <v>29</v>
+      </c>
+      <c r="F160" t="s">
+        <v>50</v>
+      </c>
+      <c r="G160" t="s">
+        <v>18</v>
+      </c>
+      <c r="H160" t="s">
+        <v>18</v>
+      </c>
+      <c r="I160" t="s">
+        <v>18</v>
+      </c>
+      <c r="J160">
+        <v>200</v>
+      </c>
+      <c r="K160">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>232</v>
+      </c>
+      <c r="B161">
+        <v>11</v>
+      </c>
+      <c r="C161" t="s">
+        <v>235</v>
+      </c>
+      <c r="D161" t="s">
+        <v>22</v>
+      </c>
+      <c r="E161" t="s">
+        <v>23</v>
+      </c>
+      <c r="F161" t="s">
+        <v>24</v>
+      </c>
+      <c r="G161" t="s">
+        <v>236</v>
+      </c>
+      <c r="H161" t="s">
+        <v>237</v>
+      </c>
+      <c r="I161" t="s">
+        <v>238</v>
+      </c>
+      <c r="J161" t="s">
+        <v>18</v>
+      </c>
+      <c r="K161" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>232</v>
+      </c>
+      <c r="B162">
+        <v>12</v>
+      </c>
+      <c r="C162" t="s">
+        <v>239</v>
+      </c>
+      <c r="D162" t="s">
+        <v>22</v>
+      </c>
+      <c r="E162" t="s">
+        <v>29</v>
+      </c>
+      <c r="F162" t="s">
+        <v>240</v>
+      </c>
+      <c r="G162" t="s">
+        <v>18</v>
+      </c>
+      <c r="H162" t="s">
+        <v>18</v>
+      </c>
+      <c r="I162" t="s">
+        <v>18</v>
+      </c>
+      <c r="J162">
+        <v>200</v>
+      </c>
+      <c r="K162">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>232</v>
+      </c>
+      <c r="B163">
+        <v>13</v>
+      </c>
+      <c r="C163" t="s">
+        <v>199</v>
+      </c>
+      <c r="D163" t="s">
+        <v>40</v>
+      </c>
+      <c r="E163" t="s">
+        <v>29</v>
+      </c>
+      <c r="F163" t="s">
+        <v>191</v>
+      </c>
+      <c r="G163" t="s">
+        <v>18</v>
+      </c>
+      <c r="H163" t="s">
+        <v>18</v>
+      </c>
+      <c r="I163" t="s">
+        <v>18</v>
+      </c>
+      <c r="J163">
+        <v>200</v>
+      </c>
+      <c r="K163">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>232</v>
+      </c>
+      <c r="B164">
+        <v>14</v>
+      </c>
+      <c r="C164" t="s">
+        <v>241</v>
+      </c>
+      <c r="D164" t="s">
+        <v>49</v>
+      </c>
+      <c r="E164" t="s">
+        <v>29</v>
+      </c>
+      <c r="F164" t="s">
+        <v>50</v>
+      </c>
+      <c r="G164" t="s">
+        <v>18</v>
+      </c>
+      <c r="H164" t="s">
+        <v>18</v>
+      </c>
+      <c r="I164" t="s">
+        <v>18</v>
+      </c>
+      <c r="J164">
+        <v>200</v>
+      </c>
+      <c r="K164">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>232</v>
+      </c>
+      <c r="B165">
+        <v>15</v>
+      </c>
+      <c r="C165" t="s">
+        <v>242</v>
+      </c>
+      <c r="D165" t="s">
+        <v>52</v>
+      </c>
+      <c r="E165" t="s">
+        <v>29</v>
+      </c>
+      <c r="F165" t="s">
+        <v>50</v>
+      </c>
+      <c r="G165" t="s">
+        <v>18</v>
+      </c>
+      <c r="H165" t="s">
+        <v>18</v>
+      </c>
+      <c r="I165" t="s">
+        <v>18</v>
+      </c>
+      <c r="J165">
+        <v>200</v>
+      </c>
+      <c r="K165">
         <v>15000</v>
       </c>
     </row>
@@ -5055,7 +7088,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E113"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -5063,10 +7096,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="C1" t="s">
-        <v>185</v>
+        <v>244</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -5086,10 +7119,10 @@
         <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E2" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -5103,10 +7136,10 @@
         <v>200</v>
       </c>
       <c r="D3" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E3" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -5120,10 +7153,10 @@
         <v>202</v>
       </c>
       <c r="D4" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E4" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -5137,10 +7170,10 @@
         <v>200</v>
       </c>
       <c r="D5" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E5" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -5154,10 +7187,10 @@
         <v>202</v>
       </c>
       <c r="D6" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E6" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -5171,10 +7204,10 @@
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E7" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -5188,10 +7221,10 @@
         <v>409</v>
       </c>
       <c r="D8" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E8" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -5205,10 +7238,10 @@
         <v>202</v>
       </c>
       <c r="D9" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E9" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -5222,10 +7255,10 @@
         <v>200</v>
       </c>
       <c r="D10" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E10" t="s">
-        <v>190</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -5239,10 +7272,10 @@
         <v>200</v>
       </c>
       <c r="D11" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E11" t="s">
-        <v>191</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5256,10 +7289,10 @@
         <v>200</v>
       </c>
       <c r="D12" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E12" t="s">
-        <v>192</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5273,10 +7306,10 @@
         <v>200</v>
       </c>
       <c r="D13" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E13" t="s">
-        <v>193</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -5290,10 +7323,10 @@
         <v>200</v>
       </c>
       <c r="D14" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E14" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -5307,10 +7340,10 @@
         <v>200</v>
       </c>
       <c r="D15" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E15" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -5324,10 +7357,10 @@
         <v>200</v>
       </c>
       <c r="D16" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E16" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -5341,10 +7374,10 @@
         <v>202</v>
       </c>
       <c r="D17" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E17" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5358,10 +7391,10 @@
         <v>200</v>
       </c>
       <c r="D18" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E18" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -5375,10 +7408,10 @@
         <v>202</v>
       </c>
       <c r="D19" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E19" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -5392,10 +7425,10 @@
         <v>200</v>
       </c>
       <c r="D20" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E20" t="s">
-        <v>195</v>
+        <v>254</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -5409,10 +7442,10 @@
         <v>200</v>
       </c>
       <c r="D21" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E21" t="s">
-        <v>196</v>
+        <v>255</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -5426,10 +7459,10 @@
         <v>200</v>
       </c>
       <c r="D22" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E22" t="s">
-        <v>197</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -5443,10 +7476,10 @@
         <v>202</v>
       </c>
       <c r="D23" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E23" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -5460,10 +7493,10 @@
         <v>200</v>
       </c>
       <c r="D24" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E24" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5477,10 +7510,10 @@
         <v>200</v>
       </c>
       <c r="D25" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E25" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -5494,10 +7527,10 @@
         <v>200</v>
       </c>
       <c r="D26" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E26" t="s">
-        <v>199</v>
+        <v>258</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -5511,10 +7544,10 @@
         <v>200</v>
       </c>
       <c r="D27" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E27" t="s">
-        <v>200</v>
+        <v>259</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -5528,10 +7561,10 @@
         <v>200</v>
       </c>
       <c r="D28" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E28" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -5545,10 +7578,10 @@
         <v>200</v>
       </c>
       <c r="D29" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E29" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -5562,10 +7595,10 @@
         <v>202</v>
       </c>
       <c r="D30" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E30" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -5579,10 +7612,10 @@
         <v>200</v>
       </c>
       <c r="D31" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E31" t="s">
-        <v>201</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -5596,10 +7629,10 @@
         <v>200</v>
       </c>
       <c r="D32" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E32" t="s">
-        <v>202</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -5613,10 +7646,10 @@
         <v>200</v>
       </c>
       <c r="D33" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E33" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -5630,10 +7663,10 @@
         <v>200</v>
       </c>
       <c r="D34" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E34" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -5647,10 +7680,10 @@
         <v>202</v>
       </c>
       <c r="D35" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E35" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -5664,10 +7697,10 @@
         <v>200</v>
       </c>
       <c r="D36" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E36" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -5681,10 +7714,10 @@
         <v>202</v>
       </c>
       <c r="D37" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E37" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -5698,10 +7731,10 @@
         <v>200</v>
       </c>
       <c r="D38" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E38" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -5715,10 +7748,10 @@
         <v>200</v>
       </c>
       <c r="D39" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E39" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -5732,10 +7765,10 @@
         <v>202</v>
       </c>
       <c r="D40" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E40" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -5749,10 +7782,10 @@
         <v>200</v>
       </c>
       <c r="D41" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E41" t="s">
-        <v>204</v>
+        <v>263</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -5766,10 +7799,10 @@
         <v>200</v>
       </c>
       <c r="D42" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E42" t="s">
-        <v>205</v>
+        <v>264</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -5783,10 +7816,10 @@
         <v>202</v>
       </c>
       <c r="D43" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E43" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -5800,10 +7833,10 @@
         <v>200</v>
       </c>
       <c r="D44" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E44" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -5817,10 +7850,10 @@
         <v>202</v>
       </c>
       <c r="D45" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E45" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -5834,10 +7867,10 @@
         <v>200</v>
       </c>
       <c r="D46" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E46" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -5851,10 +7884,10 @@
         <v>200</v>
       </c>
       <c r="D47" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E47" t="s">
-        <v>206</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -5868,10 +7901,10 @@
         <v>200</v>
       </c>
       <c r="D48" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E48" t="s">
-        <v>191</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -5885,10 +7918,10 @@
         <v>200</v>
       </c>
       <c r="D49" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E49" t="s">
-        <v>207</v>
+        <v>266</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -5902,10 +7935,10 @@
         <v>200</v>
       </c>
       <c r="D50" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E50" t="s">
-        <v>208</v>
+        <v>267</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -5919,10 +7952,10 @@
         <v>200</v>
       </c>
       <c r="D51" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E51" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -5936,10 +7969,10 @@
         <v>200</v>
       </c>
       <c r="D52" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E52" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -5953,10 +7986,10 @@
         <v>202</v>
       </c>
       <c r="D53" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E53" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -5970,10 +8003,10 @@
         <v>200</v>
       </c>
       <c r="D54" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E54" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -5987,10 +8020,10 @@
         <v>202</v>
       </c>
       <c r="D55" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E55" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -6004,10 +8037,10 @@
         <v>200</v>
       </c>
       <c r="D56" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E56" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -6021,10 +8054,10 @@
         <v>200</v>
       </c>
       <c r="D57" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E57" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -6038,10 +8071,10 @@
         <v>202</v>
       </c>
       <c r="D58" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E58" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -6055,10 +8088,10 @@
         <v>200</v>
       </c>
       <c r="D59" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E59" t="s">
-        <v>204</v>
+        <v>263</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -6072,10 +8105,10 @@
         <v>200</v>
       </c>
       <c r="D60" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E60" t="s">
-        <v>209</v>
+        <v>268</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -6089,10 +8122,10 @@
         <v>202</v>
       </c>
       <c r="D61" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E61" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -6106,10 +8139,10 @@
         <v>200</v>
       </c>
       <c r="D62" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E62" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -6123,10 +8156,10 @@
         <v>202</v>
       </c>
       <c r="D63" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E63" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -6140,10 +8173,10 @@
         <v>200</v>
       </c>
       <c r="D64" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E64" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -6157,10 +8190,10 @@
         <v>200</v>
       </c>
       <c r="D65" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E65" t="s">
-        <v>210</v>
+        <v>269</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -6174,10 +8207,10 @@
         <v>200</v>
       </c>
       <c r="D66" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E66" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -6191,10 +8224,10 @@
         <v>200</v>
       </c>
       <c r="D67" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E67" t="s">
-        <v>211</v>
+        <v>270</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -6208,10 +8241,10 @@
         <v>200</v>
       </c>
       <c r="D68" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E68" t="s">
-        <v>212</v>
+        <v>271</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -6225,10 +8258,10 @@
         <v>200</v>
       </c>
       <c r="D69" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E69" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -6242,10 +8275,10 @@
         <v>200</v>
       </c>
       <c r="D70" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E70" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -6259,10 +8292,10 @@
         <v>202</v>
       </c>
       <c r="D71" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E71" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -6276,10 +8309,10 @@
         <v>200</v>
       </c>
       <c r="D72" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E72" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -6293,10 +8326,10 @@
         <v>202</v>
       </c>
       <c r="D73" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E73" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -6310,10 +8343,10 @@
         <v>200</v>
       </c>
       <c r="D74" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E74" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -6327,10 +8360,10 @@
         <v>200</v>
       </c>
       <c r="D75" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E75" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -6344,10 +8377,10 @@
         <v>202</v>
       </c>
       <c r="D76" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E76" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -6361,10 +8394,10 @@
         <v>200</v>
       </c>
       <c r="D77" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E77" t="s">
-        <v>213</v>
+        <v>272</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -6378,10 +8411,10 @@
         <v>202</v>
       </c>
       <c r="D78" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E78" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -6395,10 +8428,10 @@
         <v>200</v>
       </c>
       <c r="D79" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E79" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -6412,10 +8445,10 @@
         <v>202</v>
       </c>
       <c r="D80" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E80" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -6429,10 +8462,10 @@
         <v>200</v>
       </c>
       <c r="D81" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E81" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -6446,10 +8479,10 @@
         <v>200</v>
       </c>
       <c r="D82" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E82" t="s">
-        <v>214</v>
+        <v>273</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -6463,10 +8496,10 @@
         <v>200</v>
       </c>
       <c r="D83" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E83" t="s">
-        <v>215</v>
+        <v>274</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -6480,10 +8513,10 @@
         <v>202</v>
       </c>
       <c r="D84" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E84" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -6497,10 +8530,10 @@
         <v>200</v>
       </c>
       <c r="D85" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E85" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -6514,10 +8547,10 @@
         <v>200</v>
       </c>
       <c r="D86" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E86" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -6531,10 +8564,10 @@
         <v>200</v>
       </c>
       <c r="D87" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E87" t="s">
-        <v>207</v>
+        <v>266</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -6548,10 +8581,10 @@
         <v>200</v>
       </c>
       <c r="D88" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E88" t="s">
-        <v>208</v>
+        <v>267</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
@@ -6565,10 +8598,10 @@
         <v>200</v>
       </c>
       <c r="D89" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E89" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -6582,10 +8615,10 @@
         <v>200</v>
       </c>
       <c r="D90" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E90" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -6599,10 +8632,10 @@
         <v>202</v>
       </c>
       <c r="D91" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E91" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -6616,10 +8649,10 @@
         <v>200</v>
       </c>
       <c r="D92" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E92" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -6633,10 +8666,10 @@
         <v>202</v>
       </c>
       <c r="D93" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E93" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -6650,10 +8683,10 @@
         <v>200</v>
       </c>
       <c r="D94" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E94" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -6667,10 +8700,10 @@
         <v>200</v>
       </c>
       <c r="D95" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E95" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -6684,10 +8717,10 @@
         <v>202</v>
       </c>
       <c r="D96" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E96" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
@@ -6701,10 +8734,10 @@
         <v>200</v>
       </c>
       <c r="D97" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E97" t="s">
-        <v>213</v>
+        <v>272</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -6718,10 +8751,10 @@
         <v>200</v>
       </c>
       <c r="D98" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E98" t="s">
-        <v>216</v>
+        <v>275</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
@@ -6735,10 +8768,10 @@
         <v>202</v>
       </c>
       <c r="D99" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E99" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -6752,10 +8785,10 @@
         <v>200</v>
       </c>
       <c r="D100" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E100" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
@@ -6769,10 +8802,10 @@
         <v>202</v>
       </c>
       <c r="D101" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E101" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
@@ -6786,10 +8819,10 @@
         <v>200</v>
       </c>
       <c r="D102" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E102" t="s">
-        <v>203</v>
+        <v>262</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
@@ -6803,10 +8836,10 @@
         <v>200</v>
       </c>
       <c r="D103" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E103" t="s">
-        <v>198</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
@@ -6820,10 +8853,10 @@
         <v>200</v>
       </c>
       <c r="D104" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E104" t="s">
-        <v>191</v>
+        <v>250</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
@@ -6837,10 +8870,10 @@
         <v>200</v>
       </c>
       <c r="D105" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E105" t="s">
-        <v>217</v>
+        <v>276</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
@@ -6854,10 +8887,10 @@
         <v>200</v>
       </c>
       <c r="D106" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E106" t="s">
-        <v>208</v>
+        <v>267</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
@@ -6871,10 +8904,10 @@
         <v>200</v>
       </c>
       <c r="D107" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E107" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -6888,10 +8921,10 @@
         <v>200</v>
       </c>
       <c r="D108" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E108" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
@@ -6905,10 +8938,10 @@
         <v>422</v>
       </c>
       <c r="D109" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E109" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
@@ -6922,10 +8955,10 @@
         <v>422</v>
       </c>
       <c r="D110" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E110" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
@@ -6939,10 +8972,10 @@
         <v>422</v>
       </c>
       <c r="D111" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E111" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
@@ -6956,10 +8989,10 @@
         <v>422</v>
       </c>
       <c r="D112" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E112" t="s">
-        <v>188</v>
+        <v>247</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
@@ -6973,10 +9006,894 @@
         <v>200</v>
       </c>
       <c r="D113" t="s">
-        <v>186</v>
+        <v>245</v>
       </c>
       <c r="E113" t="s">
-        <v>196</v>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>184</v>
+      </c>
+      <c r="B114" t="s">
+        <v>12</v>
+      </c>
+      <c r="C114">
+        <v>200</v>
+      </c>
+      <c r="D114" t="s">
+        <v>245</v>
+      </c>
+      <c r="E114" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>184</v>
+      </c>
+      <c r="B115" t="s">
+        <v>19</v>
+      </c>
+      <c r="C115">
+        <v>200</v>
+      </c>
+      <c r="D115" t="s">
+        <v>245</v>
+      </c>
+      <c r="E115" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>184</v>
+      </c>
+      <c r="B116" t="s">
+        <v>86</v>
+      </c>
+      <c r="C116">
+        <v>202</v>
+      </c>
+      <c r="D116" t="s">
+        <v>245</v>
+      </c>
+      <c r="E116" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>184</v>
+      </c>
+      <c r="B117" t="s">
+        <v>90</v>
+      </c>
+      <c r="C117">
+        <v>200</v>
+      </c>
+      <c r="D117" t="s">
+        <v>245</v>
+      </c>
+      <c r="E117" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>184</v>
+      </c>
+      <c r="B118" t="s">
+        <v>92</v>
+      </c>
+      <c r="C118">
+        <v>202</v>
+      </c>
+      <c r="D118" t="s">
+        <v>245</v>
+      </c>
+      <c r="E118" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>184</v>
+      </c>
+      <c r="B119" t="s">
+        <v>96</v>
+      </c>
+      <c r="C119">
+        <v>200</v>
+      </c>
+      <c r="D119" t="s">
+        <v>245</v>
+      </c>
+      <c r="E119" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>184</v>
+      </c>
+      <c r="B120" t="s">
+        <v>98</v>
+      </c>
+      <c r="C120">
+        <v>200</v>
+      </c>
+      <c r="D120" t="s">
+        <v>245</v>
+      </c>
+      <c r="E120" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>184</v>
+      </c>
+      <c r="B121" t="s">
+        <v>185</v>
+      </c>
+      <c r="C121">
+        <v>202</v>
+      </c>
+      <c r="D121" t="s">
+        <v>245</v>
+      </c>
+      <c r="E121" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>184</v>
+      </c>
+      <c r="B122" t="s">
+        <v>190</v>
+      </c>
+      <c r="C122">
+        <v>200</v>
+      </c>
+      <c r="D122" t="s">
+        <v>245</v>
+      </c>
+      <c r="E122" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>184</v>
+      </c>
+      <c r="B123" t="s">
+        <v>192</v>
+      </c>
+      <c r="C123">
+        <v>200</v>
+      </c>
+      <c r="D123" t="s">
+        <v>245</v>
+      </c>
+      <c r="E123" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>184</v>
+      </c>
+      <c r="B124" t="s">
+        <v>193</v>
+      </c>
+      <c r="C124">
+        <v>202</v>
+      </c>
+      <c r="D124" t="s">
+        <v>245</v>
+      </c>
+      <c r="E124" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>184</v>
+      </c>
+      <c r="B125" t="s">
+        <v>197</v>
+      </c>
+      <c r="C125">
+        <v>200</v>
+      </c>
+      <c r="D125" t="s">
+        <v>245</v>
+      </c>
+      <c r="E125" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>184</v>
+      </c>
+      <c r="B126" t="s">
+        <v>199</v>
+      </c>
+      <c r="C126">
+        <v>200</v>
+      </c>
+      <c r="D126" t="s">
+        <v>245</v>
+      </c>
+      <c r="E126" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>184</v>
+      </c>
+      <c r="B127" t="s">
+        <v>200</v>
+      </c>
+      <c r="C127">
+        <v>200</v>
+      </c>
+      <c r="D127" t="s">
+        <v>245</v>
+      </c>
+      <c r="E127" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>184</v>
+      </c>
+      <c r="B128" t="s">
+        <v>201</v>
+      </c>
+      <c r="C128">
+        <v>200</v>
+      </c>
+      <c r="D128" t="s">
+        <v>245</v>
+      </c>
+      <c r="E128" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>202</v>
+      </c>
+      <c r="B129" t="s">
+        <v>12</v>
+      </c>
+      <c r="C129">
+        <v>200</v>
+      </c>
+      <c r="D129" t="s">
+        <v>245</v>
+      </c>
+      <c r="E129" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>202</v>
+      </c>
+      <c r="B130" t="s">
+        <v>19</v>
+      </c>
+      <c r="C130">
+        <v>200</v>
+      </c>
+      <c r="D130" t="s">
+        <v>245</v>
+      </c>
+      <c r="E130" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>202</v>
+      </c>
+      <c r="B131" t="s">
+        <v>86</v>
+      </c>
+      <c r="C131">
+        <v>202</v>
+      </c>
+      <c r="D131" t="s">
+        <v>245</v>
+      </c>
+      <c r="E131" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>202</v>
+      </c>
+      <c r="B132" t="s">
+        <v>90</v>
+      </c>
+      <c r="C132">
+        <v>200</v>
+      </c>
+      <c r="D132" t="s">
+        <v>245</v>
+      </c>
+      <c r="E132" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>202</v>
+      </c>
+      <c r="B133" t="s">
+        <v>92</v>
+      </c>
+      <c r="C133">
+        <v>202</v>
+      </c>
+      <c r="D133" t="s">
+        <v>245</v>
+      </c>
+      <c r="E133" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>202</v>
+      </c>
+      <c r="B134" t="s">
+        <v>96</v>
+      </c>
+      <c r="C134">
+        <v>200</v>
+      </c>
+      <c r="D134" t="s">
+        <v>245</v>
+      </c>
+      <c r="E134" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>202</v>
+      </c>
+      <c r="B135" t="s">
+        <v>98</v>
+      </c>
+      <c r="C135">
+        <v>200</v>
+      </c>
+      <c r="D135" t="s">
+        <v>245</v>
+      </c>
+      <c r="E135" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>202</v>
+      </c>
+      <c r="B136" t="s">
+        <v>185</v>
+      </c>
+      <c r="C136">
+        <v>202</v>
+      </c>
+      <c r="D136" t="s">
+        <v>245</v>
+      </c>
+      <c r="E136" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>202</v>
+      </c>
+      <c r="B137" t="s">
+        <v>190</v>
+      </c>
+      <c r="C137">
+        <v>200</v>
+      </c>
+      <c r="D137" t="s">
+        <v>245</v>
+      </c>
+      <c r="E137" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>202</v>
+      </c>
+      <c r="B138" t="s">
+        <v>204</v>
+      </c>
+      <c r="C138">
+        <v>202</v>
+      </c>
+      <c r="D138" t="s">
+        <v>245</v>
+      </c>
+      <c r="E138" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>202</v>
+      </c>
+      <c r="B139" t="s">
+        <v>208</v>
+      </c>
+      <c r="C139">
+        <v>200</v>
+      </c>
+      <c r="D139" t="s">
+        <v>245</v>
+      </c>
+      <c r="E139" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>202</v>
+      </c>
+      <c r="B140" t="s">
+        <v>210</v>
+      </c>
+      <c r="C140">
+        <v>200</v>
+      </c>
+      <c r="D140" t="s">
+        <v>245</v>
+      </c>
+      <c r="E140" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>202</v>
+      </c>
+      <c r="B141" t="s">
+        <v>211</v>
+      </c>
+      <c r="C141">
+        <v>202</v>
+      </c>
+      <c r="D141" t="s">
+        <v>245</v>
+      </c>
+      <c r="E141" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>202</v>
+      </c>
+      <c r="B142" t="s">
+        <v>215</v>
+      </c>
+      <c r="C142">
+        <v>200</v>
+      </c>
+      <c r="D142" t="s">
+        <v>245</v>
+      </c>
+      <c r="E142" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>202</v>
+      </c>
+      <c r="B143" t="s">
+        <v>217</v>
+      </c>
+      <c r="C143">
+        <v>202</v>
+      </c>
+      <c r="D143" t="s">
+        <v>245</v>
+      </c>
+      <c r="E143" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>202</v>
+      </c>
+      <c r="B144" t="s">
+        <v>221</v>
+      </c>
+      <c r="C144">
+        <v>200</v>
+      </c>
+      <c r="D144" t="s">
+        <v>245</v>
+      </c>
+      <c r="E144" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>202</v>
+      </c>
+      <c r="B145" t="s">
+        <v>223</v>
+      </c>
+      <c r="C145">
+        <v>202</v>
+      </c>
+      <c r="D145" t="s">
+        <v>245</v>
+      </c>
+      <c r="E145" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>202</v>
+      </c>
+      <c r="B146" t="s">
+        <v>226</v>
+      </c>
+      <c r="C146">
+        <v>200</v>
+      </c>
+      <c r="D146" t="s">
+        <v>245</v>
+      </c>
+      <c r="E146" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>202</v>
+      </c>
+      <c r="B147" t="s">
+        <v>228</v>
+      </c>
+      <c r="C147">
+        <v>200</v>
+      </c>
+      <c r="D147" t="s">
+        <v>245</v>
+      </c>
+      <c r="E147" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>202</v>
+      </c>
+      <c r="B148" t="s">
+        <v>229</v>
+      </c>
+      <c r="C148">
+        <v>200</v>
+      </c>
+      <c r="D148" t="s">
+        <v>245</v>
+      </c>
+      <c r="E148" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>202</v>
+      </c>
+      <c r="B149" t="s">
+        <v>230</v>
+      </c>
+      <c r="C149">
+        <v>200</v>
+      </c>
+      <c r="D149" t="s">
+        <v>245</v>
+      </c>
+      <c r="E149" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>202</v>
+      </c>
+      <c r="B150" t="s">
+        <v>231</v>
+      </c>
+      <c r="C150">
+        <v>200</v>
+      </c>
+      <c r="D150" t="s">
+        <v>245</v>
+      </c>
+      <c r="E150" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>232</v>
+      </c>
+      <c r="B151" t="s">
+        <v>12</v>
+      </c>
+      <c r="C151">
+        <v>200</v>
+      </c>
+      <c r="D151" t="s">
+        <v>245</v>
+      </c>
+      <c r="E151" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>232</v>
+      </c>
+      <c r="B152" t="s">
+        <v>19</v>
+      </c>
+      <c r="C152">
+        <v>200</v>
+      </c>
+      <c r="D152" t="s">
+        <v>245</v>
+      </c>
+      <c r="E152" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>232</v>
+      </c>
+      <c r="B153" t="s">
+        <v>86</v>
+      </c>
+      <c r="C153">
+        <v>202</v>
+      </c>
+      <c r="D153" t="s">
+        <v>245</v>
+      </c>
+      <c r="E153" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>232</v>
+      </c>
+      <c r="B154" t="s">
+        <v>90</v>
+      </c>
+      <c r="C154">
+        <v>200</v>
+      </c>
+      <c r="D154" t="s">
+        <v>245</v>
+      </c>
+      <c r="E154" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>232</v>
+      </c>
+      <c r="B155" t="s">
+        <v>92</v>
+      </c>
+      <c r="C155">
+        <v>202</v>
+      </c>
+      <c r="D155" t="s">
+        <v>245</v>
+      </c>
+      <c r="E155" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>232</v>
+      </c>
+      <c r="B156" t="s">
+        <v>96</v>
+      </c>
+      <c r="C156">
+        <v>200</v>
+      </c>
+      <c r="D156" t="s">
+        <v>245</v>
+      </c>
+      <c r="E156" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>232</v>
+      </c>
+      <c r="B157" t="s">
+        <v>98</v>
+      </c>
+      <c r="C157">
+        <v>200</v>
+      </c>
+      <c r="D157" t="s">
+        <v>245</v>
+      </c>
+      <c r="E157" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>232</v>
+      </c>
+      <c r="B158" t="s">
+        <v>185</v>
+      </c>
+      <c r="C158">
+        <v>202</v>
+      </c>
+      <c r="D158" t="s">
+        <v>245</v>
+      </c>
+      <c r="E158" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>232</v>
+      </c>
+      <c r="B159" t="s">
+        <v>190</v>
+      </c>
+      <c r="C159">
+        <v>200</v>
+      </c>
+      <c r="D159" t="s">
+        <v>245</v>
+      </c>
+      <c r="E159" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>232</v>
+      </c>
+      <c r="B160" t="s">
+        <v>234</v>
+      </c>
+      <c r="C160">
+        <v>200</v>
+      </c>
+      <c r="D160" t="s">
+        <v>245</v>
+      </c>
+      <c r="E160" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>232</v>
+      </c>
+      <c r="B161" t="s">
+        <v>235</v>
+      </c>
+      <c r="C161">
+        <v>202</v>
+      </c>
+      <c r="D161" t="s">
+        <v>245</v>
+      </c>
+      <c r="E161" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>232</v>
+      </c>
+      <c r="B162" t="s">
+        <v>239</v>
+      </c>
+      <c r="C162">
+        <v>200</v>
+      </c>
+      <c r="D162" t="s">
+        <v>245</v>
+      </c>
+      <c r="E162" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>232</v>
+      </c>
+      <c r="B163" t="s">
+        <v>199</v>
+      </c>
+      <c r="C163">
+        <v>200</v>
+      </c>
+      <c r="D163" t="s">
+        <v>245</v>
+      </c>
+      <c r="E163" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>232</v>
+      </c>
+      <c r="B164" t="s">
+        <v>241</v>
+      </c>
+      <c r="C164">
+        <v>200</v>
+      </c>
+      <c r="D164" t="s">
+        <v>245</v>
+      </c>
+      <c r="E164" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>232</v>
+      </c>
+      <c r="B165" t="s">
+        <v>242</v>
+      </c>
+      <c r="C165">
+        <v>200</v>
+      </c>
+      <c r="D165" t="s">
+        <v>245</v>
+      </c>
+      <c r="E165" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>